<commit_message>
Remove outdated UDF specifications and prompt templates; enhance test coverage for LLM functions with a mock server; add user guide for AI/ML UDFs; update ExcelDna stubs for async functionality; adjust test script for Mono compatibility.
</commit_message>
<xml_diff>
--- a/Tests.xlsx
+++ b/Tests.xlsx
@@ -9,6 +9,8 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="AIML_Test_Data" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="AIML_UDF_Tests" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="LLM_Test_Data" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="LLM_UDF_Tests" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1" concurrentManualCount="24" forceFullCalc="1"/>
@@ -20,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000000000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -60,8 +62,13 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -95,8 +102,13 @@
         <fgColor rgb="00E7E6E6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -127,11 +139,19 @@
         <color rgb="00B7B7B7"/>
       </bottom>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="00A6A6A6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A6A6A6"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -153,6 +173,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2488,4 +2526,390 @@
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Base URL</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>http://localhost:11434</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Chat model</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>llama3.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Vision model</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>llava</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Embedding model</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>nomic-embed-text</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>API key</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sample JSON</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>{"choices":[{"message":{"content":"hello"}}]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tiny PNG Base64</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>iVBORw0KGgoAAAANSUhEUgAAAAEAAAABCAQAAAC1HAwCAAAAC0lEQVR42mP8/x8AAusB9Y9Z8xkAAAAASUVORK5CYII=</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Batch text inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>machine learning in spreadsheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>semantic search over workbook notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>cluster customer feedback</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="3" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="3" customWidth="1" min="7" max="7"/>
+    <col width="3" customWidth="1" min="8" max="8"/>
+    <col width="3" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Excel-DNA OpenAI / Ollama UDF Worksheet Harness</t>
+        </is>
+      </c>
+      <c r="B1" s="17" t="n"/>
+      <c r="C1" s="17" t="n"/>
+      <c r="D1" s="17" t="n"/>
+      <c r="E1" s="17" t="n"/>
+      <c r="F1" s="17" t="n"/>
+      <c r="G1" s="17" t="n"/>
+      <c r="H1" s="17" t="n"/>
+      <c r="I1" s="17" t="n"/>
+      <c r="J1" s="17" t="n"/>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Configure LLM_Test_Data first. Network tests show PASS after a valid endpoint/model responds; LLM_JSON_VALUE is deterministic and works offline. Async calls may briefly display #GETTING_DATA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>UDF</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>Actual formula / spill anchor</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="n"/>
+      <c r="D3" s="19" t="n"/>
+      <c r="E3" s="19" t="n"/>
+      <c r="F3" s="19" t="inlineStr">
+        <is>
+          <t>Expected / validation note</t>
+        </is>
+      </c>
+      <c r="G3" s="19" t="n"/>
+      <c r="H3" s="19" t="n"/>
+      <c r="I3" s="19" t="n"/>
+      <c r="J3" s="19">
+        <f>COUNTIF(J:J,"PASS")&amp;"/6 passed"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>LLM_CHAT</t>
+        </is>
+      </c>
+      <c r="B5" s="21">
+        <f>LLM_CHAT("Reply with exactly OK",LLM_Test_Data!B4,LLM_Test_Data!B3,LLM_Test_Data!B7,"Return only OK",0,8,LLM_Test_Data!B2)</f>
+        <v/>
+      </c>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="22" t="n"/>
+      <c r="F5" s="23" t="inlineStr">
+        <is>
+          <t>Any nonempty response without LLM_ERROR</t>
+        </is>
+      </c>
+      <c r="G5" s="22" t="n"/>
+      <c r="H5" s="22" t="n"/>
+      <c r="I5" s="22" t="n"/>
+      <c r="J5" s="24">
+        <f>IFERROR(IF(AND(B5&lt;&gt;"",LEFT(B5,10)&lt;&gt;"LLM_ERROR:"),"PASS","FAIL"),"WAIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>LLM_CHAT_IMAGE</t>
+        </is>
+      </c>
+      <c r="B10" s="21">
+        <f>LLM_CHAT_IMAGE("Describe this one-pixel image briefly",LLM_Test_Data!B9,LLM_Test_Data!B5,"image/png",LLM_Test_Data!B3,LLM_Test_Data!B7,"Be concise",0,24,LLM_Test_Data!B2)</f>
+        <v/>
+      </c>
+      <c r="C10" s="22" t="n"/>
+      <c r="D10" s="22" t="n"/>
+      <c r="E10" s="22" t="n"/>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>Any nonempty vision response without LLM_ERROR</t>
+        </is>
+      </c>
+      <c r="G10" s="22" t="n"/>
+      <c r="H10" s="22" t="n"/>
+      <c r="I10" s="22" t="n"/>
+      <c r="J10" s="24">
+        <f>IFERROR(IF(AND(B10&lt;&gt;"",LEFT(B10,10)&lt;&gt;"LLM_ERROR:"),"PASS","FAIL"),"WAIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>LLM_EMBED</t>
+        </is>
+      </c>
+      <c r="B15" s="21">
+        <f>LLM_EMBED("spreadsheet",LLM_Test_Data!B6,LLM_Test_Data!B3,LLM_Test_Data!B7,LLM_Test_Data!B2)</f>
+        <v/>
+      </c>
+      <c r="C15" s="22" t="n"/>
+      <c r="D15" s="22" t="n"/>
+      <c r="E15" s="22" t="n"/>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>Numeric vertical spill vector</t>
+        </is>
+      </c>
+      <c r="G15" s="22" t="n"/>
+      <c r="H15" s="22" t="n"/>
+      <c r="I15" s="22" t="n"/>
+      <c r="J15" s="24">
+        <f>IFERROR(IF(AND(ROWS(B15#)&gt;0,COLUMNS(B15#)=1,ISNUMBER(INDEX(B15#,1,1))),"PASS","FAIL"),"WAIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>LLM_EMBED_BATCH</t>
+        </is>
+      </c>
+      <c r="B20" s="21">
+        <f>LLM_EMBED_BATCH(LLM_Test_Data!A13:A15,LLM_Test_Data!B6,LLM_Test_Data!B3,LLM_Test_Data!B7,LLM_Test_Data!B2)</f>
+        <v/>
+      </c>
+      <c r="C20" s="22" t="n"/>
+      <c r="D20" s="22" t="n"/>
+      <c r="E20" s="22" t="n"/>
+      <c r="F20" s="23" t="inlineStr">
+        <is>
+          <t>Three embedding rows; one per input</t>
+        </is>
+      </c>
+      <c r="G20" s="22" t="n"/>
+      <c r="H20" s="22" t="n"/>
+      <c r="I20" s="22" t="n"/>
+      <c r="J20" s="24">
+        <f>IFERROR(IF(AND(ROWS(B20#)=3,COLUMNS(B20#)&gt;0,ISNUMBER(INDEX(B20#,1,1))),"PASS","FAIL"),"WAIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>LLM_LIST_MODELS</t>
+        </is>
+      </c>
+      <c r="B25" s="21">
+        <f>LLM_LIST_MODELS(LLM_Test_Data!B3,LLM_Test_Data!B7,LLM_Test_Data!B2)</f>
+        <v/>
+      </c>
+      <c r="C25" s="22" t="n"/>
+      <c r="D25" s="22" t="n"/>
+      <c r="E25" s="22" t="n"/>
+      <c r="F25" s="23" t="inlineStr">
+        <is>
+          <t>At least one model identifier</t>
+        </is>
+      </c>
+      <c r="G25" s="22" t="n"/>
+      <c r="H25" s="22" t="n"/>
+      <c r="I25" s="22" t="n"/>
+      <c r="J25" s="24">
+        <f>IFERROR(IF(AND(ROWS(B25#)&gt;0,B25&lt;&gt;""),"PASS","FAIL"),"WAIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>LLM_JSON_VALUE</t>
+        </is>
+      </c>
+      <c r="B30" s="21">
+        <f>LLM_JSON_VALUE(LLM_Test_Data!B8,"choices[0].message.content")</f>
+        <v/>
+      </c>
+      <c r="C30" s="22" t="n"/>
+      <c r="D30" s="22" t="n"/>
+      <c r="E30" s="22" t="n"/>
+      <c r="F30" s="23" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="G30" s="22" t="n"/>
+      <c r="H30" s="22" t="n"/>
+      <c r="I30" s="22" t="n"/>
+      <c r="J30" s="24">
+        <f>IFERROR(IF(B30=F30,"PASS","FAIL"),"FAIL")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>